<commit_message>
Add Profiler3 network correlation analysis
</commit_message>
<xml_diff>
--- a/CaImg Python/results/profiler1_summary.xlsx
+++ b/CaImg Python/results/profiler1_summary.xlsx
@@ -445,10 +445,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C2" t="n">
-        <v>784</v>
+        <v>859</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
@@ -461,10 +461,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C3" t="n">
-        <v>825</v>
+        <v>913</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
@@ -477,10 +477,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>826</v>
+        <v>898</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
@@ -493,10 +493,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C5" t="n">
-        <v>802</v>
+        <v>888</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
@@ -509,10 +509,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C6" t="n">
-        <v>908</v>
+        <v>1016</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
@@ -525,13 +525,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>990</v>
+        <v>1099</v>
       </c>
       <c r="D7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -541,10 +541,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C8" t="n">
-        <v>873</v>
+        <v>983</v>
       </c>
       <c r="D8" t="b">
         <v>1</v>
@@ -560,7 +560,7 @@
         <v>17</v>
       </c>
       <c r="C9" t="n">
-        <v>832</v>
+        <v>959</v>
       </c>
       <c r="D9" t="b">
         <v>1</v>
@@ -573,10 +573,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C10" t="n">
-        <v>808</v>
+        <v>900</v>
       </c>
       <c r="D10" t="b">
         <v>1</v>
@@ -589,10 +589,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" t="n">
-        <v>857</v>
+        <v>968</v>
       </c>
       <c r="D11" t="b">
         <v>1</v>
@@ -605,10 +605,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C12" t="n">
-        <v>893</v>
+        <v>1059</v>
       </c>
       <c r="D12" t="b">
         <v>1</v>
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>975</v>
+        <v>1099</v>
       </c>
       <c r="D13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -653,10 +653,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C15" t="n">
-        <v>811</v>
+        <v>893</v>
       </c>
       <c r="D15" t="b">
         <v>1</v>
@@ -669,10 +669,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C16" t="n">
-        <v>769</v>
+        <v>844</v>
       </c>
       <c r="D16" t="b">
         <v>1</v>
@@ -685,10 +685,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C17" t="n">
-        <v>823</v>
+        <v>911</v>
       </c>
       <c r="D17" t="b">
         <v>1</v>
@@ -701,10 +701,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>940</v>
+        <v>1013</v>
       </c>
       <c r="D18" t="b">
         <v>1</v>
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C19" t="n">
-        <v>935</v>
+        <v>1055</v>
       </c>
       <c r="D19" t="b">
         <v>1</v>
@@ -733,10 +733,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C20" t="n">
-        <v>895</v>
+        <v>1040</v>
       </c>
       <c r="D20" t="b">
         <v>1</v>
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C21" t="n">
-        <v>882</v>
+        <v>989</v>
       </c>
       <c r="D21" t="b">
         <v>1</v>
@@ -765,10 +765,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C22" t="n">
-        <v>867</v>
+        <v>972</v>
       </c>
       <c r="D22" t="b">
         <v>1</v>
@@ -781,10 +781,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C23" t="n">
-        <v>729</v>
+        <v>811</v>
       </c>
       <c r="D23" t="b">
         <v>1</v>
@@ -797,10 +797,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C24" t="n">
-        <v>821</v>
+        <v>898</v>
       </c>
       <c r="D24" t="b">
         <v>1</v>
@@ -813,10 +813,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C25" t="n">
-        <v>829</v>
+        <v>910</v>
       </c>
       <c r="D25" t="b">
         <v>1</v>
@@ -829,10 +829,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C26" t="n">
-        <v>877</v>
+        <v>957</v>
       </c>
       <c r="D26" t="b">
         <v>1</v>
@@ -845,10 +845,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C27" t="n">
-        <v>825</v>
+        <v>891</v>
       </c>
       <c r="D27" t="b">
         <v>1</v>
@@ -864,7 +864,7 @@
         <v>17</v>
       </c>
       <c r="C28" t="n">
-        <v>746</v>
+        <v>819</v>
       </c>
       <c r="D28" t="b">
         <v>1</v>
@@ -877,10 +877,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C29" t="n">
-        <v>783</v>
+        <v>852</v>
       </c>
       <c r="D29" t="b">
         <v>1</v>
@@ -896,7 +896,7 @@
         <v>20</v>
       </c>
       <c r="C30" t="n">
-        <v>854</v>
+        <v>929</v>
       </c>
       <c r="D30" t="b">
         <v>1</v>
@@ -909,10 +909,10 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C31" t="n">
-        <v>771</v>
+        <v>852</v>
       </c>
       <c r="D31" t="b">
         <v>1</v>
@@ -925,10 +925,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C32" t="n">
-        <v>784</v>
+        <v>871</v>
       </c>
       <c r="D32" t="b">
         <v>1</v>
@@ -944,7 +944,7 @@
         <v>17</v>
       </c>
       <c r="C33" t="n">
-        <v>736</v>
+        <v>807</v>
       </c>
       <c r="D33" t="b">
         <v>1</v>
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C34" t="n">
-        <v>901</v>
+        <v>1019</v>
       </c>
       <c r="D34" t="b">
         <v>1</v>
@@ -973,13 +973,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>973</v>
+        <v>1099</v>
       </c>
       <c r="D35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -989,10 +989,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C36" t="n">
-        <v>887</v>
+        <v>972</v>
       </c>
       <c r="D36" t="b">
         <v>1</v>
@@ -1005,10 +1005,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C37" t="n">
-        <v>835</v>
+        <v>938</v>
       </c>
       <c r="D37" t="b">
         <v>1</v>
@@ -1021,10 +1021,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C38" t="n">
-        <v>936</v>
+        <v>1035</v>
       </c>
       <c r="D38" t="b">
         <v>1</v>
@@ -1053,13 +1053,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C40" t="n">
-        <v>899</v>
+        <v>1093</v>
       </c>
       <c r="D40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1069,13 +1069,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C41" t="n">
-        <v>996</v>
+        <v>1099</v>
       </c>
       <c r="D41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -1085,13 +1085,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C42" t="n">
-        <v>1038</v>
+        <v>1099</v>
       </c>
       <c r="D42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -1101,10 +1101,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C43" t="n">
-        <v>857</v>
+        <v>984</v>
       </c>
       <c r="D43" t="b">
         <v>1</v>
@@ -1117,13 +1117,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>992</v>
+        <v>1099</v>
       </c>
       <c r="D44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -1133,13 +1133,13 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C45" t="n">
-        <v>937</v>
+        <v>1099</v>
       </c>
       <c r="D45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -1149,10 +1149,10 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C46" t="n">
-        <v>886</v>
+        <v>1074</v>
       </c>
       <c r="D46" t="b">
         <v>1</v>
@@ -1165,10 +1165,10 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C47" t="n">
-        <v>898</v>
+        <v>991</v>
       </c>
       <c r="D47" t="b">
         <v>1</v>
@@ -1181,10 +1181,10 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C48" t="n">
-        <v>954</v>
+        <v>1045</v>
       </c>
       <c r="D48" t="b">
         <v>1</v>
@@ -1197,13 +1197,13 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>939</v>
+        <v>1099</v>
       </c>
       <c r="D49" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -1213,13 +1213,13 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C50" t="n">
-        <v>941</v>
+        <v>1099</v>
       </c>
       <c r="D50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -1229,10 +1229,10 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="C51" t="n">
-        <v>949</v>
+        <v>1086</v>
       </c>
       <c r="D51" t="b">
         <v>1</v>
@@ -1248,7 +1248,7 @@
         <v>17</v>
       </c>
       <c r="C52" t="n">
-        <v>711</v>
+        <v>803</v>
       </c>
       <c r="D52" t="b">
         <v>1</v>
@@ -1261,10 +1261,10 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C53" t="n">
-        <v>820</v>
+        <v>914</v>
       </c>
       <c r="D53" t="b">
         <v>1</v>
@@ -1277,10 +1277,10 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C54" t="n">
-        <v>887</v>
+        <v>985</v>
       </c>
       <c r="D54" t="b">
         <v>1</v>
@@ -1293,10 +1293,10 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C55" t="n">
-        <v>837</v>
+        <v>926</v>
       </c>
       <c r="D55" t="b">
         <v>1</v>
@@ -1309,10 +1309,10 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C56" t="n">
-        <v>907</v>
+        <v>1019</v>
       </c>
       <c r="D56" t="b">
         <v>1</v>
@@ -1325,10 +1325,10 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C57" t="n">
-        <v>860</v>
+        <v>935</v>
       </c>
       <c r="D57" t="b">
         <v>1</v>
@@ -1344,7 +1344,7 @@
         <v>20</v>
       </c>
       <c r="C58" t="n">
-        <v>874</v>
+        <v>938</v>
       </c>
       <c r="D58" t="b">
         <v>1</v>
@@ -1360,7 +1360,7 @@
         <v>20</v>
       </c>
       <c r="C59" t="n">
-        <v>877</v>
+        <v>958</v>
       </c>
       <c r="D59" t="b">
         <v>1</v>
@@ -1373,10 +1373,10 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="C60" t="n">
-        <v>944</v>
+        <v>1064</v>
       </c>
       <c r="D60" t="b">
         <v>1</v>
@@ -1392,7 +1392,7 @@
         <v>20</v>
       </c>
       <c r="C61" t="n">
-        <v>880</v>
+        <v>950</v>
       </c>
       <c r="D61" t="b">
         <v>1</v>
@@ -1405,10 +1405,10 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C62" t="n">
-        <v>796</v>
+        <v>859</v>
       </c>
       <c r="D62" t="b">
         <v>1</v>
@@ -1421,10 +1421,10 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C63" t="n">
-        <v>835</v>
+        <v>905</v>
       </c>
       <c r="D63" t="b">
         <v>1</v>
@@ -1440,7 +1440,7 @@
         <v>20</v>
       </c>
       <c r="C64" t="n">
-        <v>893</v>
+        <v>950</v>
       </c>
       <c r="D64" t="b">
         <v>1</v>
@@ -1456,7 +1456,7 @@
         <v>20</v>
       </c>
       <c r="C65" t="n">
-        <v>871</v>
+        <v>936</v>
       </c>
       <c r="D65" t="b">
         <v>1</v>
@@ -1469,10 +1469,10 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C66" t="n">
-        <v>857</v>
+        <v>926</v>
       </c>
       <c r="D66" t="b">
         <v>1</v>
@@ -1485,10 +1485,10 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C67" t="n">
-        <v>834</v>
+        <v>927</v>
       </c>
       <c r="D67" t="b">
         <v>1</v>
@@ -1501,10 +1501,10 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C68" t="n">
-        <v>822</v>
+        <v>906</v>
       </c>
       <c r="D68" t="b">
         <v>1</v>
@@ -1517,10 +1517,10 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C69" t="n">
-        <v>906</v>
+        <v>970</v>
       </c>
       <c r="D69" t="b">
         <v>1</v>
@@ -1533,10 +1533,10 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C70" t="n">
-        <v>886</v>
+        <v>1010</v>
       </c>
       <c r="D70" t="b">
         <v>1</v>
@@ -1549,10 +1549,10 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C71" t="n">
-        <v>899</v>
+        <v>968</v>
       </c>
       <c r="D71" t="b">
         <v>1</v>
@@ -1565,10 +1565,10 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C72" t="n">
-        <v>911</v>
+        <v>980</v>
       </c>
       <c r="D72" t="b">
         <v>1</v>
@@ -1581,10 +1581,10 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C73" t="n">
-        <v>859</v>
+        <v>927</v>
       </c>
       <c r="D73" t="b">
         <v>1</v>
@@ -1600,7 +1600,7 @@
         <v>20</v>
       </c>
       <c r="C74" t="n">
-        <v>887</v>
+        <v>951</v>
       </c>
       <c r="D74" t="b">
         <v>1</v>
@@ -1613,10 +1613,10 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C75" t="n">
-        <v>919</v>
+        <v>988</v>
       </c>
       <c r="D75" t="b">
         <v>1</v>
@@ -1629,13 +1629,13 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C76" t="n">
-        <v>950</v>
+        <v>1086</v>
       </c>
       <c r="D76" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -1645,10 +1645,10 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C77" t="n">
-        <v>892</v>
+        <v>971</v>
       </c>
       <c r="D77" t="b">
         <v>1</v>
@@ -1664,7 +1664,7 @@
         <v>20</v>
       </c>
       <c r="C78" t="n">
-        <v>902</v>
+        <v>976</v>
       </c>
       <c r="D78" t="b">
         <v>1</v>
@@ -1677,10 +1677,10 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C79" t="n">
-        <v>862</v>
+        <v>949</v>
       </c>
       <c r="D79" t="b">
         <v>1</v>
@@ -1693,10 +1693,10 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C80" t="n">
-        <v>911</v>
+        <v>1023</v>
       </c>
       <c r="D80" t="b">
         <v>1</v>
@@ -1709,10 +1709,10 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C81" t="n">
-        <v>871</v>
+        <v>1032</v>
       </c>
       <c r="D81" t="b">
         <v>1</v>
@@ -1725,13 +1725,13 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="C82" t="n">
-        <v>974</v>
+        <v>1092</v>
       </c>
       <c r="D82" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -1741,13 +1741,13 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="C83" t="n">
-        <v>991</v>
+        <v>1099</v>
       </c>
       <c r="D83" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -1757,13 +1757,13 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C84" t="n">
-        <v>1010</v>
+        <v>1099</v>
       </c>
       <c r="D84" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -1776,7 +1776,7 @@
         <v>17</v>
       </c>
       <c r="C85" t="n">
-        <v>772</v>
+        <v>868</v>
       </c>
       <c r="D85" t="b">
         <v>1</v>
@@ -1789,10 +1789,10 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C86" t="n">
-        <v>777</v>
+        <v>875</v>
       </c>
       <c r="D86" t="b">
         <v>1</v>
@@ -1805,13 +1805,13 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C87" t="n">
-        <v>915</v>
+        <v>1099</v>
       </c>
       <c r="D87" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -1821,10 +1821,10 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C88" t="n">
-        <v>885</v>
+        <v>970</v>
       </c>
       <c r="D88" t="b">
         <v>1</v>
@@ -1840,7 +1840,7 @@
         <v>19</v>
       </c>
       <c r="C89" t="n">
-        <v>862</v>
+        <v>973</v>
       </c>
       <c r="D89" t="b">
         <v>1</v>
@@ -1853,10 +1853,10 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C90" t="n">
-        <v>906</v>
+        <v>1015</v>
       </c>
       <c r="D90" t="b">
         <v>1</v>
@@ -1869,13 +1869,13 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="C91" t="n">
-        <v>993</v>
+        <v>1099</v>
       </c>
       <c r="D91" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -1885,13 +1885,13 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C92" t="n">
-        <v>1018</v>
+        <v>1099</v>
       </c>
       <c r="D92" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -1901,10 +1901,10 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C93" t="n">
-        <v>881</v>
+        <v>968</v>
       </c>
       <c r="D93" t="b">
         <v>1</v>
@@ -1917,10 +1917,10 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C94" t="n">
-        <v>960</v>
+        <v>1050</v>
       </c>
       <c r="D94" t="b">
         <v>1</v>
@@ -1933,10 +1933,10 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C95" t="n">
-        <v>875</v>
+        <v>930</v>
       </c>
       <c r="D95" t="b">
         <v>1</v>
@@ -1965,13 +1965,13 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="C97" t="n">
-        <v>972</v>
+        <v>1099</v>
       </c>
       <c r="D97" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C98" t="n">
-        <v>785</v>
+        <v>865</v>
       </c>
       <c r="D98" t="b">
         <v>1</v>
@@ -1997,10 +1997,10 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C99" t="n">
-        <v>793</v>
+        <v>871</v>
       </c>
       <c r="D99" t="b">
         <v>1</v>
@@ -2013,10 +2013,10 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C100" t="n">
-        <v>953</v>
+        <v>1044</v>
       </c>
       <c r="D100" t="b">
         <v>1</v>
@@ -2029,10 +2029,10 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C101" t="n">
-        <v>926</v>
+        <v>1017</v>
       </c>
       <c r="D101" t="b">
         <v>1</v>

</xml_diff>